<commit_message>
fix: changes as per review
</commit_message>
<xml_diff>
--- a/india_compliance/gst_india/data/test_gstr2b_export_golden.xlsx
+++ b/india_compliance/gst_india/data/test_gstr2b_export_golden.xlsx
@@ -11206,6 +11206,21 @@
           <t>No</t>
         </is>
       </c>
+      <c r="I7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>Nov'19</t>
@@ -11582,6 +11597,21 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="K8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="46" t="n">
+        <v>0</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -12884,6 +12914,21 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="O7" t="inlineStr">
         <is>
           <t>Nov'19</t>
@@ -13290,6 +13335,21 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="N8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="46" t="n">
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>

</xml_diff>